<commit_message>
ui: move strikeouts to end of batting; logo+name-only compare dropdown; lighter team boxes
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/data/mlb_team_stats.xlsx
+++ b/docs/data/mlb_team_stats.xlsx
@@ -450,52 +450,52 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Runs Rank</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Home Runs</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Home Runs Rank</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>On-Base %</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>On-Base % Rank</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Slugging %</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Slugging % Rank</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Batting Strikeouts</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Batting Strikeouts Rank</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Runs</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Runs Rank</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Home Runs</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Home Runs Rank</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>On-Base %</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>On-Base % Rank</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Slugging %</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Slugging % Rank</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
@@ -552,34 +552,34 @@
         <v>22</v>
       </c>
       <c r="D2" t="n">
+        <v>331</v>
+      </c>
+      <c r="E2" t="n">
+        <v>17</v>
+      </c>
+      <c r="F2" t="n">
+        <v>68</v>
+      </c>
+      <c r="G2" t="n">
+        <v>27</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.3089631</v>
+      </c>
+      <c r="I2" t="n">
+        <v>26</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.38401255</v>
+      </c>
+      <c r="K2" t="n">
+        <v>25</v>
+      </c>
+      <c r="L2" t="n">
         <v>569</v>
       </c>
-      <c r="E2" t="n">
+      <c r="M2" t="n">
         <v>3</v>
-      </c>
-      <c r="F2" t="n">
-        <v>331</v>
-      </c>
-      <c r="G2" t="n">
-        <v>17</v>
-      </c>
-      <c r="H2" t="n">
-        <v>68</v>
-      </c>
-      <c r="I2" t="n">
-        <v>27</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.3089631</v>
-      </c>
-      <c r="K2" t="n">
-        <v>26</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.38401255</v>
-      </c>
-      <c r="M2" t="n">
-        <v>25</v>
       </c>
       <c r="N2" t="n">
         <v>4.3035803</v>
@@ -619,34 +619,34 @@
         <v>8</v>
       </c>
       <c r="D3" t="n">
+        <v>364</v>
+      </c>
+      <c r="E3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F3" t="n">
+        <v>105</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.32978722</v>
+      </c>
+      <c r="I3" t="n">
+        <v>7</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.42038217</v>
+      </c>
+      <c r="K3" t="n">
+        <v>5</v>
+      </c>
+      <c r="L3" t="n">
         <v>672</v>
       </c>
-      <c r="E3" t="n">
+      <c r="M3" t="n">
         <v>24</v>
-      </c>
-      <c r="F3" t="n">
-        <v>364</v>
-      </c>
-      <c r="G3" t="n">
-        <v>10</v>
-      </c>
-      <c r="H3" t="n">
-        <v>105</v>
-      </c>
-      <c r="I3" t="n">
-        <v>3</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.32978722</v>
-      </c>
-      <c r="K3" t="n">
-        <v>7</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.42038217</v>
-      </c>
-      <c r="M3" t="n">
-        <v>5</v>
       </c>
       <c r="N3" t="n">
         <v>4.999048</v>
@@ -686,34 +686,34 @@
         <v>6</v>
       </c>
       <c r="D4" t="n">
+        <v>377</v>
+      </c>
+      <c r="E4" t="n">
+        <v>7</v>
+      </c>
+      <c r="F4" t="n">
+        <v>101</v>
+      </c>
+      <c r="G4" t="n">
+        <v>6</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.316655</v>
+      </c>
+      <c r="I4" t="n">
+        <v>19</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.42109343</v>
+      </c>
+      <c r="K4" t="n">
+        <v>4</v>
+      </c>
+      <c r="L4" t="n">
         <v>604</v>
       </c>
-      <c r="E4" t="n">
+      <c r="M4" t="n">
         <v>6</v>
-      </c>
-      <c r="F4" t="n">
-        <v>377</v>
-      </c>
-      <c r="G4" t="n">
-        <v>7</v>
-      </c>
-      <c r="H4" t="n">
-        <v>101</v>
-      </c>
-      <c r="I4" t="n">
-        <v>6</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.316655</v>
-      </c>
-      <c r="K4" t="n">
-        <v>19</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.42109343</v>
-      </c>
-      <c r="M4" t="n">
-        <v>4</v>
       </c>
       <c r="N4" t="n">
         <v>3.404926</v>
@@ -753,34 +753,34 @@
         <v>20</v>
       </c>
       <c r="D5" t="n">
-        <v>714</v>
+        <v>369</v>
       </c>
       <c r="E5" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
       <c r="F5" t="n">
-        <v>369</v>
+        <v>94</v>
       </c>
       <c r="G5" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="H5" t="n">
-        <v>94</v>
+        <v>0.3213807</v>
       </c>
       <c r="I5" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="J5" t="n">
-        <v>0.3213807</v>
+        <v>0.4030303</v>
       </c>
       <c r="K5" t="n">
         <v>12</v>
       </c>
       <c r="L5" t="n">
-        <v>0.4030303</v>
+        <v>714</v>
       </c>
       <c r="M5" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="N5" t="n">
         <v>4.4549356</v>
@@ -820,34 +820,34 @@
         <v>18</v>
       </c>
       <c r="D6" t="n">
+        <v>294</v>
+      </c>
+      <c r="E6" t="n">
+        <v>30</v>
+      </c>
+      <c r="F6" t="n">
+        <v>64</v>
+      </c>
+      <c r="G6" t="n">
+        <v>29</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.31099963</v>
+      </c>
+      <c r="I6" t="n">
+        <v>25</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.38061184</v>
+      </c>
+      <c r="K6" t="n">
+        <v>27</v>
+      </c>
+      <c r="L6" t="n">
         <v>628</v>
       </c>
-      <c r="E6" t="n">
+      <c r="M6" t="n">
         <v>11</v>
-      </c>
-      <c r="F6" t="n">
-        <v>294</v>
-      </c>
-      <c r="G6" t="n">
-        <v>30</v>
-      </c>
-      <c r="H6" t="n">
-        <v>64</v>
-      </c>
-      <c r="I6" t="n">
-        <v>29</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.31099963</v>
-      </c>
-      <c r="K6" t="n">
-        <v>25</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.38061184</v>
-      </c>
-      <c r="M6" t="n">
-        <v>27</v>
       </c>
       <c r="N6" t="n">
         <v>3.8513105</v>
@@ -887,34 +887,34 @@
         <v>16</v>
       </c>
       <c r="D7" t="n">
+        <v>366</v>
+      </c>
+      <c r="E7" t="n">
+        <v>9</v>
+      </c>
+      <c r="F7" t="n">
+        <v>90</v>
+      </c>
+      <c r="G7" t="n">
+        <v>15</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.33707866</v>
+      </c>
+      <c r="I7" t="n">
+        <v>3</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.40129572</v>
+      </c>
+      <c r="K7" t="n">
+        <v>14</v>
+      </c>
+      <c r="L7" t="n">
         <v>636</v>
       </c>
-      <c r="E7" t="n">
+      <c r="M7" t="n">
         <v>13</v>
-      </c>
-      <c r="F7" t="n">
-        <v>366</v>
-      </c>
-      <c r="G7" t="n">
-        <v>9</v>
-      </c>
-      <c r="H7" t="n">
-        <v>90</v>
-      </c>
-      <c r="I7" t="n">
-        <v>15</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.33707866</v>
-      </c>
-      <c r="K7" t="n">
-        <v>3</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.40129572</v>
-      </c>
-      <c r="M7" t="n">
-        <v>14</v>
       </c>
       <c r="N7" t="n">
         <v>4.280488</v>
@@ -954,34 +954,34 @@
         <v>23</v>
       </c>
       <c r="D8" t="n">
+        <v>353</v>
+      </c>
+      <c r="E8" t="n">
+        <v>14</v>
+      </c>
+      <c r="F8" t="n">
+        <v>106</v>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.3189776</v>
+      </c>
+      <c r="I8" t="n">
+        <v>16</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.40982956</v>
+      </c>
+      <c r="K8" t="n">
+        <v>9</v>
+      </c>
+      <c r="L8" t="n">
         <v>692</v>
       </c>
-      <c r="E8" t="n">
+      <c r="M8" t="n">
         <v>26</v>
-      </c>
-      <c r="F8" t="n">
-        <v>353</v>
-      </c>
-      <c r="G8" t="n">
-        <v>14</v>
-      </c>
-      <c r="H8" t="n">
-        <v>106</v>
-      </c>
-      <c r="I8" t="n">
-        <v>2</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.3189776</v>
-      </c>
-      <c r="K8" t="n">
-        <v>16</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.40982956</v>
-      </c>
-      <c r="M8" t="n">
-        <v>9</v>
       </c>
       <c r="N8" t="n">
         <v>4.408437</v>
@@ -1021,34 +1021,34 @@
         <v>28</v>
       </c>
       <c r="D9" t="n">
+        <v>325</v>
+      </c>
+      <c r="E9" t="n">
+        <v>22</v>
+      </c>
+      <c r="F9" t="n">
+        <v>96</v>
+      </c>
+      <c r="G9" t="n">
+        <v>11</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.31135023</v>
+      </c>
+      <c r="I9" t="n">
+        <v>24</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.39498433</v>
+      </c>
+      <c r="K9" t="n">
+        <v>18</v>
+      </c>
+      <c r="L9" t="n">
         <v>712</v>
       </c>
-      <c r="E9" t="n">
+      <c r="M9" t="n">
         <v>27</v>
-      </c>
-      <c r="F9" t="n">
-        <v>325</v>
-      </c>
-      <c r="G9" t="n">
-        <v>22</v>
-      </c>
-      <c r="H9" t="n">
-        <v>96</v>
-      </c>
-      <c r="I9" t="n">
-        <v>11</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0.31135023</v>
-      </c>
-      <c r="K9" t="n">
-        <v>24</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.39498433</v>
-      </c>
-      <c r="M9" t="n">
-        <v>18</v>
       </c>
       <c r="N9" t="n">
         <v>4.579646</v>
@@ -1088,34 +1088,34 @@
         <v>29</v>
       </c>
       <c r="D10" t="n">
+        <v>310</v>
+      </c>
+      <c r="E10" t="n">
+        <v>27</v>
+      </c>
+      <c r="F10" t="n">
+        <v>74</v>
+      </c>
+      <c r="G10" t="n">
+        <v>25</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.3125</v>
+      </c>
+      <c r="I10" t="n">
+        <v>22</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.3702544</v>
+      </c>
+      <c r="K10" t="n">
+        <v>29</v>
+      </c>
+      <c r="L10" t="n">
         <v>627</v>
       </c>
-      <c r="E10" t="n">
+      <c r="M10" t="n">
         <v>10</v>
-      </c>
-      <c r="F10" t="n">
-        <v>310</v>
-      </c>
-      <c r="G10" t="n">
-        <v>27</v>
-      </c>
-      <c r="H10" t="n">
-        <v>74</v>
-      </c>
-      <c r="I10" t="n">
-        <v>25</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.3125</v>
-      </c>
-      <c r="K10" t="n">
-        <v>22</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.3702544</v>
-      </c>
-      <c r="M10" t="n">
-        <v>29</v>
       </c>
       <c r="N10" t="n">
         <v>3.7917676</v>
@@ -1155,34 +1155,34 @@
         <v>7</v>
       </c>
       <c r="D11" t="n">
+        <v>356</v>
+      </c>
+      <c r="E11" t="n">
+        <v>12</v>
+      </c>
+      <c r="F11" t="n">
+        <v>84</v>
+      </c>
+      <c r="G11" t="n">
+        <v>18</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.3224822</v>
+      </c>
+      <c r="I11" t="n">
+        <v>11</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.4096933</v>
+      </c>
+      <c r="K11" t="n">
+        <v>10</v>
+      </c>
+      <c r="L11" t="n">
         <v>687</v>
       </c>
-      <c r="E11" t="n">
+      <c r="M11" t="n">
         <v>25</v>
-      </c>
-      <c r="F11" t="n">
-        <v>356</v>
-      </c>
-      <c r="G11" t="n">
-        <v>12</v>
-      </c>
-      <c r="H11" t="n">
-        <v>84</v>
-      </c>
-      <c r="I11" t="n">
-        <v>18</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0.3224822</v>
-      </c>
-      <c r="K11" t="n">
-        <v>11</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.4096933</v>
-      </c>
-      <c r="M11" t="n">
-        <v>10</v>
       </c>
       <c r="N11" t="n">
         <v>5.5263157</v>
@@ -1222,34 +1222,34 @@
         <v>24</v>
       </c>
       <c r="D12" t="n">
-        <v>664</v>
+        <v>314</v>
       </c>
       <c r="E12" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="F12" t="n">
-        <v>314</v>
+        <v>86</v>
       </c>
       <c r="G12" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="H12" t="n">
-        <v>86</v>
+        <v>0.31471202</v>
       </c>
       <c r="I12" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="J12" t="n">
-        <v>0.31471202</v>
+        <v>0.39333335</v>
       </c>
       <c r="K12" t="n">
         <v>20</v>
       </c>
       <c r="L12" t="n">
-        <v>0.39333335</v>
+        <v>664</v>
       </c>
       <c r="M12" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="N12" t="n">
         <v>3.8342404</v>
@@ -1289,34 +1289,34 @@
         <v>17</v>
       </c>
       <c r="D13" t="n">
+        <v>356</v>
+      </c>
+      <c r="E13" t="n">
+        <v>12</v>
+      </c>
+      <c r="F13" t="n">
+        <v>103</v>
+      </c>
+      <c r="G13" t="n">
+        <v>5</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.31749243</v>
+      </c>
+      <c r="I13" t="n">
+        <v>18</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.41251886</v>
+      </c>
+      <c r="K13" t="n">
+        <v>7</v>
+      </c>
+      <c r="L13" t="n">
         <v>647</v>
       </c>
-      <c r="E13" t="n">
+      <c r="M13" t="n">
         <v>17</v>
-      </c>
-      <c r="F13" t="n">
-        <v>356</v>
-      </c>
-      <c r="G13" t="n">
-        <v>12</v>
-      </c>
-      <c r="H13" t="n">
-        <v>103</v>
-      </c>
-      <c r="I13" t="n">
-        <v>5</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0.31749243</v>
-      </c>
-      <c r="K13" t="n">
-        <v>18</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.41251886</v>
-      </c>
-      <c r="M13" t="n">
-        <v>7</v>
       </c>
       <c r="N13" t="n">
         <v>4.839866</v>
@@ -1356,34 +1356,34 @@
         <v>11</v>
       </c>
       <c r="D14" t="n">
+        <v>331</v>
+      </c>
+      <c r="E14" t="n">
+        <v>17</v>
+      </c>
+      <c r="F14" t="n">
+        <v>77</v>
+      </c>
+      <c r="G14" t="n">
+        <v>23</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.32111338</v>
+      </c>
+      <c r="I14" t="n">
+        <v>13</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.39518902</v>
+      </c>
+      <c r="K14" t="n">
+        <v>17</v>
+      </c>
+      <c r="L14" t="n">
         <v>616</v>
       </c>
-      <c r="E14" t="n">
+      <c r="M14" t="n">
         <v>9</v>
-      </c>
-      <c r="F14" t="n">
-        <v>331</v>
-      </c>
-      <c r="G14" t="n">
-        <v>17</v>
-      </c>
-      <c r="H14" t="n">
-        <v>77</v>
-      </c>
-      <c r="I14" t="n">
-        <v>23</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0.32111338</v>
-      </c>
-      <c r="K14" t="n">
-        <v>13</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.39518902</v>
-      </c>
-      <c r="M14" t="n">
-        <v>17</v>
       </c>
       <c r="N14" t="n">
         <v>4.5760503</v>
@@ -1423,34 +1423,34 @@
         <v>21</v>
       </c>
       <c r="D15" t="n">
-        <v>747</v>
+        <v>361</v>
       </c>
       <c r="E15" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="F15" t="n">
-        <v>361</v>
+        <v>95</v>
       </c>
       <c r="G15" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H15" t="n">
-        <v>95</v>
+        <v>0.31977326</v>
       </c>
       <c r="I15" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="J15" t="n">
-        <v>0.31977326</v>
+        <v>0.40105143</v>
       </c>
       <c r="K15" t="n">
         <v>15</v>
       </c>
       <c r="L15" t="n">
-        <v>0.40105143</v>
+        <v>747</v>
       </c>
       <c r="M15" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="N15" t="n">
         <v>4.6507177</v>
@@ -1490,34 +1490,34 @@
         <v>1</v>
       </c>
       <c r="D16" t="n">
+        <v>405</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" t="n">
+        <v>105</v>
+      </c>
+      <c r="G16" t="n">
+        <v>3</v>
+      </c>
+      <c r="H16" t="n">
+        <v>0.34316355</v>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0.43536633</v>
+      </c>
+      <c r="K16" t="n">
+        <v>2</v>
+      </c>
+      <c r="L16" t="n">
         <v>615</v>
       </c>
-      <c r="E16" t="n">
+      <c r="M16" t="n">
         <v>8</v>
-      </c>
-      <c r="F16" t="n">
-        <v>405</v>
-      </c>
-      <c r="G16" t="n">
-        <v>2</v>
-      </c>
-      <c r="H16" t="n">
-        <v>105</v>
-      </c>
-      <c r="I16" t="n">
-        <v>3</v>
-      </c>
-      <c r="J16" t="n">
-        <v>0.34316355</v>
-      </c>
-      <c r="K16" t="n">
-        <v>1</v>
-      </c>
-      <c r="L16" t="n">
-        <v>0.43536633</v>
-      </c>
-      <c r="M16" t="n">
-        <v>2</v>
       </c>
       <c r="N16" t="n">
         <v>3.4568381</v>
@@ -1557,34 +1557,34 @@
         <v>15</v>
       </c>
       <c r="D17" t="n">
+        <v>336</v>
+      </c>
+      <c r="E17" t="n">
+        <v>16</v>
+      </c>
+      <c r="F17" t="n">
+        <v>69</v>
+      </c>
+      <c r="G17" t="n">
+        <v>26</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.32289156</v>
+      </c>
+      <c r="I17" t="n">
+        <v>10</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.38677043</v>
+      </c>
+      <c r="K17" t="n">
+        <v>24</v>
+      </c>
+      <c r="L17" t="n">
         <v>641</v>
       </c>
-      <c r="E17" t="n">
+      <c r="M17" t="n">
         <v>15</v>
-      </c>
-      <c r="F17" t="n">
-        <v>336</v>
-      </c>
-      <c r="G17" t="n">
-        <v>16</v>
-      </c>
-      <c r="H17" t="n">
-        <v>69</v>
-      </c>
-      <c r="I17" t="n">
-        <v>26</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0.32289156</v>
-      </c>
-      <c r="K17" t="n">
-        <v>10</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0.38677043</v>
-      </c>
-      <c r="M17" t="n">
-        <v>24</v>
       </c>
       <c r="N17" t="n">
         <v>4.072993</v>
@@ -1624,34 +1624,34 @@
         <v>4</v>
       </c>
       <c r="D18" t="n">
+        <v>397</v>
+      </c>
+      <c r="E18" t="n">
+        <v>3</v>
+      </c>
+      <c r="F18" t="n">
+        <v>68</v>
+      </c>
+      <c r="G18" t="n">
+        <v>27</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.33999312</v>
+      </c>
+      <c r="I18" t="n">
+        <v>2</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.39357114</v>
+      </c>
+      <c r="K18" t="n">
+        <v>19</v>
+      </c>
+      <c r="L18" t="n">
         <v>610</v>
       </c>
-      <c r="E18" t="n">
+      <c r="M18" t="n">
         <v>7</v>
-      </c>
-      <c r="F18" t="n">
-        <v>397</v>
-      </c>
-      <c r="G18" t="n">
-        <v>3</v>
-      </c>
-      <c r="H18" t="n">
-        <v>68</v>
-      </c>
-      <c r="I18" t="n">
-        <v>27</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0.33999312</v>
-      </c>
-      <c r="K18" t="n">
-        <v>2</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0.39357114</v>
-      </c>
-      <c r="M18" t="n">
-        <v>19</v>
       </c>
       <c r="N18" t="n">
         <v>3.4488072</v>
@@ -1691,34 +1691,34 @@
         <v>12</v>
       </c>
       <c r="D19" t="n">
+        <v>388</v>
+      </c>
+      <c r="E19" t="n">
+        <v>6</v>
+      </c>
+      <c r="F19" t="n">
+        <v>97</v>
+      </c>
+      <c r="G19" t="n">
+        <v>10</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0.32345104</v>
+      </c>
+      <c r="I19" t="n">
+        <v>9</v>
+      </c>
+      <c r="J19" t="n">
+        <v>0.4117647</v>
+      </c>
+      <c r="K19" t="n">
+        <v>8</v>
+      </c>
+      <c r="L19" t="n">
         <v>657</v>
       </c>
-      <c r="E19" t="n">
+      <c r="M19" t="n">
         <v>19</v>
-      </c>
-      <c r="F19" t="n">
-        <v>388</v>
-      </c>
-      <c r="G19" t="n">
-        <v>6</v>
-      </c>
-      <c r="H19" t="n">
-        <v>97</v>
-      </c>
-      <c r="I19" t="n">
-        <v>10</v>
-      </c>
-      <c r="J19" t="n">
-        <v>0.32345104</v>
-      </c>
-      <c r="K19" t="n">
-        <v>9</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0.4117647</v>
-      </c>
-      <c r="M19" t="n">
-        <v>8</v>
       </c>
       <c r="N19" t="n">
         <v>4.78907</v>
@@ -1758,34 +1758,34 @@
         <v>26</v>
       </c>
       <c r="D20" t="n">
+        <v>311</v>
+      </c>
+      <c r="E20" t="n">
+        <v>26</v>
+      </c>
+      <c r="F20" t="n">
+        <v>82</v>
+      </c>
+      <c r="G20" t="n">
+        <v>19</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.29722124</v>
+      </c>
+      <c r="I20" t="n">
+        <v>29</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.37199378</v>
+      </c>
+      <c r="K20" t="n">
+        <v>28</v>
+      </c>
+      <c r="L20" t="n">
         <v>638</v>
       </c>
-      <c r="E20" t="n">
+      <c r="M20" t="n">
         <v>14</v>
-      </c>
-      <c r="F20" t="n">
-        <v>311</v>
-      </c>
-      <c r="G20" t="n">
-        <v>26</v>
-      </c>
-      <c r="H20" t="n">
-        <v>82</v>
-      </c>
-      <c r="I20" t="n">
-        <v>19</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0.29722124</v>
-      </c>
-      <c r="K20" t="n">
-        <v>29</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0.37199378</v>
-      </c>
-      <c r="M20" t="n">
-        <v>28</v>
       </c>
       <c r="N20" t="n">
         <v>4.08932</v>
@@ -1825,34 +1825,34 @@
         <v>14</v>
       </c>
       <c r="D21" t="n">
+        <v>389</v>
+      </c>
+      <c r="E21" t="n">
+        <v>5</v>
+      </c>
+      <c r="F21" t="n">
+        <v>114</v>
+      </c>
+      <c r="G21" t="n">
+        <v>1</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.33159903</v>
+      </c>
+      <c r="I21" t="n">
+        <v>6</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.43863815</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1</v>
+      </c>
+      <c r="L21" t="n">
         <v>657</v>
       </c>
-      <c r="E21" t="n">
+      <c r="M21" t="n">
         <v>19</v>
-      </c>
-      <c r="F21" t="n">
-        <v>389</v>
-      </c>
-      <c r="G21" t="n">
-        <v>5</v>
-      </c>
-      <c r="H21" t="n">
-        <v>114</v>
-      </c>
-      <c r="I21" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0.33159903</v>
-      </c>
-      <c r="K21" t="n">
-        <v>6</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0.43863815</v>
-      </c>
-      <c r="M21" t="n">
-        <v>1</v>
       </c>
       <c r="N21" t="n">
         <v>3.3450148</v>
@@ -1892,34 +1892,34 @@
         <v>25</v>
       </c>
       <c r="D22" t="n">
+        <v>329</v>
+      </c>
+      <c r="E22" t="n">
+        <v>19</v>
+      </c>
+      <c r="F22" t="n">
+        <v>99</v>
+      </c>
+      <c r="G22" t="n">
+        <v>8</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.30031502</v>
+      </c>
+      <c r="I22" t="n">
+        <v>28</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.39643136</v>
+      </c>
+      <c r="K22" t="n">
+        <v>16</v>
+      </c>
+      <c r="L22" t="n">
         <v>660</v>
       </c>
-      <c r="E22" t="n">
+      <c r="M22" t="n">
         <v>21</v>
-      </c>
-      <c r="F22" t="n">
-        <v>329</v>
-      </c>
-      <c r="G22" t="n">
-        <v>19</v>
-      </c>
-      <c r="H22" t="n">
-        <v>99</v>
-      </c>
-      <c r="I22" t="n">
-        <v>8</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0.30031502</v>
-      </c>
-      <c r="K22" t="n">
-        <v>28</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0.39643136</v>
-      </c>
-      <c r="M22" t="n">
-        <v>16</v>
       </c>
       <c r="N22" t="n">
         <v>4.0578794</v>
@@ -1959,34 +1959,34 @@
         <v>5</v>
       </c>
       <c r="D23" t="n">
+        <v>391</v>
+      </c>
+      <c r="E23" t="n">
+        <v>4</v>
+      </c>
+      <c r="F23" t="n">
+        <v>94</v>
+      </c>
+      <c r="G23" t="n">
+        <v>13</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.33464438</v>
+      </c>
+      <c r="I23" t="n">
+        <v>4</v>
+      </c>
+      <c r="J23" t="n">
+        <v>0.40925926</v>
+      </c>
+      <c r="K23" t="n">
+        <v>11</v>
+      </c>
+      <c r="L23" t="n">
         <v>720</v>
       </c>
-      <c r="E23" t="n">
+      <c r="M23" t="n">
         <v>29</v>
-      </c>
-      <c r="F23" t="n">
-        <v>391</v>
-      </c>
-      <c r="G23" t="n">
-        <v>4</v>
-      </c>
-      <c r="H23" t="n">
-        <v>94</v>
-      </c>
-      <c r="I23" t="n">
-        <v>13</v>
-      </c>
-      <c r="J23" t="n">
-        <v>0.33464438</v>
-      </c>
-      <c r="K23" t="n">
-        <v>4</v>
-      </c>
-      <c r="L23" t="n">
-        <v>0.40925926</v>
-      </c>
-      <c r="M23" t="n">
-        <v>11</v>
       </c>
       <c r="N23" t="n">
         <v>4.2123094</v>
@@ -2026,34 +2026,34 @@
         <v>30</v>
       </c>
       <c r="D24" t="n">
-        <v>645</v>
+        <v>296</v>
       </c>
       <c r="E24" t="n">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F24" t="n">
-        <v>296</v>
+        <v>78</v>
       </c>
       <c r="G24" t="n">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="H24" t="n">
-        <v>78</v>
+        <v>0.29252437</v>
       </c>
       <c r="I24" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="J24" t="n">
-        <v>0.29252437</v>
+        <v>0.36389223</v>
       </c>
       <c r="K24" t="n">
         <v>30</v>
       </c>
       <c r="L24" t="n">
-        <v>0.36389223</v>
+        <v>645</v>
       </c>
       <c r="M24" t="n">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="N24" t="n">
         <v>3.9049034</v>
@@ -2093,34 +2093,34 @@
         <v>2</v>
       </c>
       <c r="D25" t="n">
+        <v>317</v>
+      </c>
+      <c r="E25" t="n">
+        <v>23</v>
+      </c>
+      <c r="F25" t="n">
+        <v>81</v>
+      </c>
+      <c r="G25" t="n">
+        <v>20</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.30878285</v>
+      </c>
+      <c r="I25" t="n">
+        <v>27</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.41857842</v>
+      </c>
+      <c r="K25" t="n">
+        <v>6</v>
+      </c>
+      <c r="L25" t="n">
         <v>592</v>
       </c>
-      <c r="E25" t="n">
+      <c r="M25" t="n">
         <v>5</v>
-      </c>
-      <c r="F25" t="n">
-        <v>317</v>
-      </c>
-      <c r="G25" t="n">
-        <v>23</v>
-      </c>
-      <c r="H25" t="n">
-        <v>81</v>
-      </c>
-      <c r="I25" t="n">
-        <v>20</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0.30878285</v>
-      </c>
-      <c r="K25" t="n">
-        <v>27</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0.41857842</v>
-      </c>
-      <c r="M25" t="n">
-        <v>6</v>
       </c>
       <c r="N25" t="n">
         <v>4.4624815</v>
@@ -2160,34 +2160,34 @@
         <v>27</v>
       </c>
       <c r="D26" t="n">
+        <v>326</v>
+      </c>
+      <c r="E26" t="n">
+        <v>21</v>
+      </c>
+      <c r="F26" t="n">
+        <v>98</v>
+      </c>
+      <c r="G26" t="n">
+        <v>9</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.31254238</v>
+      </c>
+      <c r="I26" t="n">
+        <v>21</v>
+      </c>
+      <c r="J26" t="n">
+        <v>0.38714615</v>
+      </c>
+      <c r="K26" t="n">
+        <v>22</v>
+      </c>
+      <c r="L26" t="n">
         <v>669</v>
       </c>
-      <c r="E26" t="n">
+      <c r="M26" t="n">
         <v>23</v>
-      </c>
-      <c r="F26" t="n">
-        <v>326</v>
-      </c>
-      <c r="G26" t="n">
-        <v>21</v>
-      </c>
-      <c r="H26" t="n">
-        <v>98</v>
-      </c>
-      <c r="I26" t="n">
-        <v>9</v>
-      </c>
-      <c r="J26" t="n">
-        <v>0.31254238</v>
-      </c>
-      <c r="K26" t="n">
-        <v>21</v>
-      </c>
-      <c r="L26" t="n">
-        <v>0.38714615</v>
-      </c>
-      <c r="M26" t="n">
-        <v>22</v>
       </c>
       <c r="N26" t="n">
         <v>3.623044</v>
@@ -2227,34 +2227,34 @@
         <v>9</v>
       </c>
       <c r="D27" t="n">
+        <v>349</v>
+      </c>
+      <c r="E27" t="n">
+        <v>15</v>
+      </c>
+      <c r="F27" t="n">
+        <v>87</v>
+      </c>
+      <c r="G27" t="n">
+        <v>16</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.32752612</v>
+      </c>
+      <c r="I27" t="n">
+        <v>8</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.4016555</v>
+      </c>
+      <c r="K27" t="n">
+        <v>13</v>
+      </c>
+      <c r="L27" t="n">
         <v>587</v>
       </c>
-      <c r="E27" t="n">
+      <c r="M27" t="n">
         <v>4</v>
-      </c>
-      <c r="F27" t="n">
-        <v>349</v>
-      </c>
-      <c r="G27" t="n">
-        <v>15</v>
-      </c>
-      <c r="H27" t="n">
-        <v>87</v>
-      </c>
-      <c r="I27" t="n">
-        <v>16</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0.32752612</v>
-      </c>
-      <c r="K27" t="n">
-        <v>8</v>
-      </c>
-      <c r="L27" t="n">
-        <v>0.4016555</v>
-      </c>
-      <c r="M27" t="n">
-        <v>13</v>
       </c>
       <c r="N27" t="n">
         <v>4.2942348</v>
@@ -2294,34 +2294,34 @@
         <v>3</v>
       </c>
       <c r="D28" t="n">
+        <v>327</v>
+      </c>
+      <c r="E28" t="n">
+        <v>20</v>
+      </c>
+      <c r="F28" t="n">
+        <v>62</v>
+      </c>
+      <c r="G28" t="n">
+        <v>30</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.33416727</v>
+      </c>
+      <c r="I28" t="n">
+        <v>5</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.38312474</v>
+      </c>
+      <c r="K28" t="n">
+        <v>26</v>
+      </c>
+      <c r="L28" t="n">
         <v>540</v>
       </c>
-      <c r="E28" t="n">
+      <c r="M28" t="n">
         <v>1</v>
-      </c>
-      <c r="F28" t="n">
-        <v>327</v>
-      </c>
-      <c r="G28" t="n">
-        <v>20</v>
-      </c>
-      <c r="H28" t="n">
-        <v>62</v>
-      </c>
-      <c r="I28" t="n">
-        <v>30</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0.33416727</v>
-      </c>
-      <c r="K28" t="n">
-        <v>5</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0.38312474</v>
-      </c>
-      <c r="M28" t="n">
-        <v>26</v>
       </c>
       <c r="N28" t="n">
         <v>3.9077156</v>
@@ -2361,34 +2361,34 @@
         <v>19</v>
       </c>
       <c r="D29" t="n">
+        <v>309</v>
+      </c>
+      <c r="E29" t="n">
+        <v>28</v>
+      </c>
+      <c r="F29" t="n">
+        <v>78</v>
+      </c>
+      <c r="G29" t="n">
+        <v>21</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.31778628</v>
+      </c>
+      <c r="I29" t="n">
+        <v>17</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.3869582</v>
+      </c>
+      <c r="K29" t="n">
+        <v>23</v>
+      </c>
+      <c r="L29" t="n">
         <v>652</v>
       </c>
-      <c r="E29" t="n">
+      <c r="M29" t="n">
         <v>18</v>
-      </c>
-      <c r="F29" t="n">
-        <v>309</v>
-      </c>
-      <c r="G29" t="n">
-        <v>28</v>
-      </c>
-      <c r="H29" t="n">
-        <v>78</v>
-      </c>
-      <c r="I29" t="n">
-        <v>21</v>
-      </c>
-      <c r="J29" t="n">
-        <v>0.31778628</v>
-      </c>
-      <c r="K29" t="n">
-        <v>17</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0.3869582</v>
-      </c>
-      <c r="M29" t="n">
-        <v>23</v>
       </c>
       <c r="N29" t="n">
         <v>3.9447186</v>
@@ -2428,34 +2428,34 @@
         <v>10</v>
       </c>
       <c r="D30" t="n">
-        <v>562</v>
+        <v>316</v>
       </c>
       <c r="E30" t="n">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="F30" t="n">
-        <v>316</v>
+        <v>77</v>
       </c>
       <c r="G30" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H30" t="n">
-        <v>77</v>
+        <v>0.31138355</v>
       </c>
       <c r="I30" t="n">
         <v>23</v>
       </c>
       <c r="J30" t="n">
-        <v>0.31138355</v>
+        <v>0.39133796</v>
       </c>
       <c r="K30" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="L30" t="n">
-        <v>0.39133796</v>
+        <v>562</v>
       </c>
       <c r="M30" t="n">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="N30" t="n">
         <v>4.1325183</v>
@@ -2495,34 +2495,34 @@
         <v>13</v>
       </c>
       <c r="D31" t="n">
+        <v>416</v>
+      </c>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="n">
+        <v>101</v>
+      </c>
+      <c r="G31" t="n">
+        <v>6</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.3204698</v>
+      </c>
+      <c r="I31" t="n">
+        <v>14</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.42123032</v>
+      </c>
+      <c r="K31" t="n">
+        <v>3</v>
+      </c>
+      <c r="L31" t="n">
         <v>631</v>
       </c>
-      <c r="E31" t="n">
+      <c r="M31" t="n">
         <v>12</v>
-      </c>
-      <c r="F31" t="n">
-        <v>416</v>
-      </c>
-      <c r="G31" t="n">
-        <v>1</v>
-      </c>
-      <c r="H31" t="n">
-        <v>101</v>
-      </c>
-      <c r="I31" t="n">
-        <v>6</v>
-      </c>
-      <c r="J31" t="n">
-        <v>0.3204698</v>
-      </c>
-      <c r="K31" t="n">
-        <v>14</v>
-      </c>
-      <c r="L31" t="n">
-        <v>0.42123032</v>
-      </c>
-      <c r="M31" t="n">
-        <v>3</v>
       </c>
       <c r="N31" t="n">
         <v>4.6370125</v>
@@ -2704,52 +2704,52 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>Runs</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Runs Rank</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Home Runs</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Home Runs Rank</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>On-Base %</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>On-Base % Rank</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Slugging %</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Slugging % Rank</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
           <t>Batting Strikeouts</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Batting Strikeouts Rank</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Runs</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>Runs Rank</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>Home Runs</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>Home Runs Rank</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>On-Base %</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>On-Base % Rank</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Slugging %</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>Slugging % Rank</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
@@ -2806,34 +2806,34 @@
         <v>13</v>
       </c>
       <c r="D2" t="n">
+        <v>31</v>
+      </c>
+      <c r="E2" t="n">
+        <v>9</v>
+      </c>
+      <c r="F2" t="n">
+        <v>4</v>
+      </c>
+      <c r="G2" t="n">
+        <v>28</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.33777776</v>
+      </c>
+      <c r="I2" t="n">
+        <v>7</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.37688443</v>
+      </c>
+      <c r="K2" t="n">
+        <v>24</v>
+      </c>
+      <c r="L2" t="n">
         <v>32</v>
       </c>
-      <c r="E2" t="n">
+      <c r="M2" t="n">
         <v>2</v>
-      </c>
-      <c r="F2" t="n">
-        <v>31</v>
-      </c>
-      <c r="G2" t="n">
-        <v>9</v>
-      </c>
-      <c r="H2" t="n">
-        <v>4</v>
-      </c>
-      <c r="I2" t="n">
-        <v>28</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.33777776</v>
-      </c>
-      <c r="K2" t="n">
-        <v>7</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.37688443</v>
-      </c>
-      <c r="M2" t="n">
-        <v>24</v>
       </c>
       <c r="N2" t="n">
         <v>5.6666665</v>
@@ -2873,34 +2873,34 @@
         <v>14</v>
       </c>
       <c r="D3" t="n">
-        <v>67</v>
+        <v>44</v>
       </c>
       <c r="E3" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>44</v>
+        <v>13</v>
       </c>
       <c r="G3" t="n">
         <v>2</v>
       </c>
       <c r="H3" t="n">
-        <v>13</v>
+        <v>0.33576643</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="J3" t="n">
-        <v>0.33576643</v>
+        <v>0.4625</v>
       </c>
       <c r="K3" t="n">
         <v>8</v>
       </c>
       <c r="L3" t="n">
-        <v>0.4625</v>
+        <v>67</v>
       </c>
       <c r="M3" t="n">
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="N3" t="n">
         <v>6.46875</v>
@@ -2940,34 +2940,34 @@
         <v>20</v>
       </c>
       <c r="D4" t="n">
+        <v>18</v>
+      </c>
+      <c r="E4" t="n">
+        <v>28</v>
+      </c>
+      <c r="F4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G4" t="n">
+        <v>21</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.26704547</v>
+      </c>
+      <c r="I4" t="n">
+        <v>26</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.37951806</v>
+      </c>
+      <c r="K4" t="n">
+        <v>22</v>
+      </c>
+      <c r="L4" t="n">
         <v>48</v>
       </c>
-      <c r="E4" t="n">
+      <c r="M4" t="n">
         <v>13</v>
-      </c>
-      <c r="F4" t="n">
-        <v>18</v>
-      </c>
-      <c r="G4" t="n">
-        <v>28</v>
-      </c>
-      <c r="H4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I4" t="n">
-        <v>21</v>
-      </c>
-      <c r="J4" t="n">
-        <v>0.26704547</v>
-      </c>
-      <c r="K4" t="n">
-        <v>26</v>
-      </c>
-      <c r="L4" t="n">
-        <v>0.37951806</v>
-      </c>
-      <c r="M4" t="n">
-        <v>22</v>
       </c>
       <c r="N4" t="n">
         <v>5</v>
@@ -3007,34 +3007,34 @@
         <v>26</v>
       </c>
       <c r="D5" t="n">
+        <v>26</v>
+      </c>
+      <c r="E5" t="n">
+        <v>14</v>
+      </c>
+      <c r="F5" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" t="n">
+        <v>12</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.2882883</v>
+      </c>
+      <c r="I5" t="n">
+        <v>23</v>
+      </c>
+      <c r="J5" t="n">
+        <v>0.38916257</v>
+      </c>
+      <c r="K5" t="n">
+        <v>19</v>
+      </c>
+      <c r="L5" t="n">
         <v>62</v>
       </c>
-      <c r="E5" t="n">
+      <c r="M5" t="n">
         <v>27</v>
-      </c>
-      <c r="F5" t="n">
-        <v>26</v>
-      </c>
-      <c r="G5" t="n">
-        <v>14</v>
-      </c>
-      <c r="H5" t="n">
-        <v>8</v>
-      </c>
-      <c r="I5" t="n">
-        <v>12</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0.2882883</v>
-      </c>
-      <c r="K5" t="n">
-        <v>23</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0.38916257</v>
-      </c>
-      <c r="M5" t="n">
-        <v>19</v>
       </c>
       <c r="N5" t="n">
         <v>2.7870967</v>
@@ -3074,34 +3074,34 @@
         <v>27</v>
       </c>
       <c r="D6" t="n">
+        <v>16</v>
+      </c>
+      <c r="E6" t="n">
+        <v>29</v>
+      </c>
+      <c r="F6" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>21</v>
+      </c>
+      <c r="H6" t="n">
+        <v>0.2824074</v>
+      </c>
+      <c r="I6" t="n">
+        <v>25</v>
+      </c>
+      <c r="J6" t="n">
+        <v>0.34358975</v>
+      </c>
+      <c r="K6" t="n">
+        <v>29</v>
+      </c>
+      <c r="L6" t="n">
         <v>59</v>
       </c>
-      <c r="E6" t="n">
+      <c r="M6" t="n">
         <v>25</v>
-      </c>
-      <c r="F6" t="n">
-        <v>16</v>
-      </c>
-      <c r="G6" t="n">
-        <v>29</v>
-      </c>
-      <c r="H6" t="n">
-        <v>6</v>
-      </c>
-      <c r="I6" t="n">
-        <v>21</v>
-      </c>
-      <c r="J6" t="n">
-        <v>0.2824074</v>
-      </c>
-      <c r="K6" t="n">
-        <v>25</v>
-      </c>
-      <c r="L6" t="n">
-        <v>0.34358975</v>
-      </c>
-      <c r="M6" t="n">
-        <v>29</v>
       </c>
       <c r="N6" t="n">
         <v>3.2264152</v>
@@ -3141,34 +3141,34 @@
         <v>3</v>
       </c>
       <c r="D7" t="n">
+        <v>37</v>
+      </c>
+      <c r="E7" t="n">
+        <v>6</v>
+      </c>
+      <c r="F7" t="n">
+        <v>7</v>
+      </c>
+      <c r="G7" t="n">
+        <v>16</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0.42465752</v>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0.5222222</v>
+      </c>
+      <c r="K7" t="n">
+        <v>4</v>
+      </c>
+      <c r="L7" t="n">
         <v>33</v>
       </c>
-      <c r="E7" t="n">
+      <c r="M7" t="n">
         <v>3</v>
-      </c>
-      <c r="F7" t="n">
-        <v>37</v>
-      </c>
-      <c r="G7" t="n">
-        <v>6</v>
-      </c>
-      <c r="H7" t="n">
-        <v>7</v>
-      </c>
-      <c r="I7" t="n">
-        <v>16</v>
-      </c>
-      <c r="J7" t="n">
-        <v>0.42465752</v>
-      </c>
-      <c r="K7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0.5222222</v>
-      </c>
-      <c r="M7" t="n">
-        <v>4</v>
       </c>
       <c r="N7" t="n">
         <v>5</v>
@@ -3208,31 +3208,31 @@
         <v>28</v>
       </c>
       <c r="D8" t="n">
+        <v>20</v>
+      </c>
+      <c r="E8" t="n">
+        <v>25</v>
+      </c>
+      <c r="F8" t="n">
+        <v>10</v>
+      </c>
+      <c r="G8" t="n">
+        <v>7</v>
+      </c>
+      <c r="H8" t="n">
+        <v>0.24651162</v>
+      </c>
+      <c r="I8" t="n">
+        <v>30</v>
+      </c>
+      <c r="J8" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="K8" t="n">
+        <v>21</v>
+      </c>
+      <c r="L8" t="n">
         <v>57</v>
-      </c>
-      <c r="E8" t="n">
-        <v>21</v>
-      </c>
-      <c r="F8" t="n">
-        <v>20</v>
-      </c>
-      <c r="G8" t="n">
-        <v>25</v>
-      </c>
-      <c r="H8" t="n">
-        <v>10</v>
-      </c>
-      <c r="I8" t="n">
-        <v>7</v>
-      </c>
-      <c r="J8" t="n">
-        <v>0.24651162</v>
-      </c>
-      <c r="K8" t="n">
-        <v>30</v>
-      </c>
-      <c r="L8" t="n">
-        <v>0.38</v>
       </c>
       <c r="M8" t="n">
         <v>21</v>
@@ -3275,34 +3275,34 @@
         <v>24</v>
       </c>
       <c r="D9" t="n">
+        <v>32</v>
+      </c>
+      <c r="E9" t="n">
+        <v>7</v>
+      </c>
+      <c r="F9" t="n">
+        <v>7</v>
+      </c>
+      <c r="G9" t="n">
+        <v>16</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0.30357143</v>
+      </c>
+      <c r="I9" t="n">
+        <v>20</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0.415</v>
+      </c>
+      <c r="K9" t="n">
+        <v>16</v>
+      </c>
+      <c r="L9" t="n">
         <v>61</v>
       </c>
-      <c r="E9" t="n">
+      <c r="M9" t="n">
         <v>26</v>
-      </c>
-      <c r="F9" t="n">
-        <v>32</v>
-      </c>
-      <c r="G9" t="n">
-        <v>7</v>
-      </c>
-      <c r="H9" t="n">
-        <v>7</v>
-      </c>
-      <c r="I9" t="n">
-        <v>16</v>
-      </c>
-      <c r="J9" t="n">
-        <v>0.30357143</v>
-      </c>
-      <c r="K9" t="n">
-        <v>20</v>
-      </c>
-      <c r="L9" t="n">
-        <v>0.415</v>
-      </c>
-      <c r="M9" t="n">
-        <v>16</v>
       </c>
       <c r="N9" t="n">
         <v>3.3962264</v>
@@ -3342,34 +3342,34 @@
         <v>29</v>
       </c>
       <c r="D10" t="n">
+        <v>21</v>
+      </c>
+      <c r="E10" t="n">
+        <v>23</v>
+      </c>
+      <c r="F10" t="n">
+        <v>8</v>
+      </c>
+      <c r="G10" t="n">
+        <v>12</v>
+      </c>
+      <c r="H10" t="n">
+        <v>0.25943395</v>
+      </c>
+      <c r="I10" t="n">
+        <v>29</v>
+      </c>
+      <c r="J10" t="n">
+        <v>0.34895834</v>
+      </c>
+      <c r="K10" t="n">
+        <v>28</v>
+      </c>
+      <c r="L10" t="n">
         <v>69</v>
       </c>
-      <c r="E10" t="n">
+      <c r="M10" t="n">
         <v>30</v>
-      </c>
-      <c r="F10" t="n">
-        <v>21</v>
-      </c>
-      <c r="G10" t="n">
-        <v>23</v>
-      </c>
-      <c r="H10" t="n">
-        <v>8</v>
-      </c>
-      <c r="I10" t="n">
-        <v>12</v>
-      </c>
-      <c r="J10" t="n">
-        <v>0.25943395</v>
-      </c>
-      <c r="K10" t="n">
-        <v>29</v>
-      </c>
-      <c r="L10" t="n">
-        <v>0.34895834</v>
-      </c>
-      <c r="M10" t="n">
-        <v>28</v>
       </c>
       <c r="N10" t="n">
         <v>4.32</v>
@@ -3409,34 +3409,34 @@
         <v>23</v>
       </c>
       <c r="D11" t="n">
+        <v>27</v>
+      </c>
+      <c r="E11" t="n">
+        <v>12</v>
+      </c>
+      <c r="F11" t="n">
+        <v>9</v>
+      </c>
+      <c r="G11" t="n">
+        <v>9</v>
+      </c>
+      <c r="H11" t="n">
+        <v>0.32568806</v>
+      </c>
+      <c r="I11" t="n">
+        <v>13</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0.41361257</v>
+      </c>
+      <c r="K11" t="n">
+        <v>17</v>
+      </c>
+      <c r="L11" t="n">
         <v>42</v>
       </c>
-      <c r="E11" t="n">
+      <c r="M11" t="n">
         <v>9</v>
-      </c>
-      <c r="F11" t="n">
-        <v>27</v>
-      </c>
-      <c r="G11" t="n">
-        <v>12</v>
-      </c>
-      <c r="H11" t="n">
-        <v>9</v>
-      </c>
-      <c r="I11" t="n">
-        <v>9</v>
-      </c>
-      <c r="J11" t="n">
-        <v>0.32568806</v>
-      </c>
-      <c r="K11" t="n">
-        <v>13</v>
-      </c>
-      <c r="L11" t="n">
-        <v>0.41361257</v>
-      </c>
-      <c r="M11" t="n">
-        <v>17</v>
       </c>
       <c r="N11" t="n">
         <v>4.5</v>
@@ -3476,34 +3476,34 @@
         <v>18</v>
       </c>
       <c r="D12" t="n">
+        <v>26</v>
+      </c>
+      <c r="E12" t="n">
+        <v>14</v>
+      </c>
+      <c r="F12" t="n">
+        <v>10</v>
+      </c>
+      <c r="G12" t="n">
+        <v>7</v>
+      </c>
+      <c r="H12" t="n">
+        <v>0.3105023</v>
+      </c>
+      <c r="I12" t="n">
+        <v>18</v>
+      </c>
+      <c r="J12" t="n">
+        <v>0.4314721</v>
+      </c>
+      <c r="K12" t="n">
+        <v>12</v>
+      </c>
+      <c r="L12" t="n">
         <v>57</v>
       </c>
-      <c r="E12" t="n">
+      <c r="M12" t="n">
         <v>21</v>
-      </c>
-      <c r="F12" t="n">
-        <v>26</v>
-      </c>
-      <c r="G12" t="n">
-        <v>14</v>
-      </c>
-      <c r="H12" t="n">
-        <v>10</v>
-      </c>
-      <c r="I12" t="n">
-        <v>7</v>
-      </c>
-      <c r="J12" t="n">
-        <v>0.3105023</v>
-      </c>
-      <c r="K12" t="n">
-        <v>18</v>
-      </c>
-      <c r="L12" t="n">
-        <v>0.4314721</v>
-      </c>
-      <c r="M12" t="n">
-        <v>12</v>
       </c>
       <c r="N12" t="n">
         <v>2.54717</v>
@@ -3543,34 +3543,34 @@
         <v>12</v>
       </c>
       <c r="D13" t="n">
+        <v>23</v>
+      </c>
+      <c r="E13" t="n">
+        <v>20</v>
+      </c>
+      <c r="F13" t="n">
+        <v>7</v>
+      </c>
+      <c r="G13" t="n">
+        <v>16</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0.31132075</v>
+      </c>
+      <c r="I13" t="n">
+        <v>17</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0.43076923</v>
+      </c>
+      <c r="K13" t="n">
+        <v>13</v>
+      </c>
+      <c r="L13" t="n">
         <v>47</v>
       </c>
-      <c r="E13" t="n">
+      <c r="M13" t="n">
         <v>12</v>
-      </c>
-      <c r="F13" t="n">
-        <v>23</v>
-      </c>
-      <c r="G13" t="n">
-        <v>20</v>
-      </c>
-      <c r="H13" t="n">
-        <v>7</v>
-      </c>
-      <c r="I13" t="n">
-        <v>16</v>
-      </c>
-      <c r="J13" t="n">
-        <v>0.31132075</v>
-      </c>
-      <c r="K13" t="n">
-        <v>17</v>
-      </c>
-      <c r="L13" t="n">
-        <v>0.43076923</v>
-      </c>
-      <c r="M13" t="n">
-        <v>13</v>
       </c>
       <c r="N13" t="n">
         <v>4</v>
@@ -3610,34 +3610,34 @@
         <v>2</v>
       </c>
       <c r="D14" t="n">
+        <v>43</v>
+      </c>
+      <c r="E14" t="n">
+        <v>4</v>
+      </c>
+      <c r="F14" t="n">
+        <v>13</v>
+      </c>
+      <c r="G14" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.375</v>
+      </c>
+      <c r="I14" t="n">
+        <v>4</v>
+      </c>
+      <c r="J14" t="n">
+        <v>0.58064514</v>
+      </c>
+      <c r="K14" t="n">
+        <v>1</v>
+      </c>
+      <c r="L14" t="n">
         <v>38</v>
       </c>
-      <c r="E14" t="n">
+      <c r="M14" t="n">
         <v>7</v>
-      </c>
-      <c r="F14" t="n">
-        <v>43</v>
-      </c>
-      <c r="G14" t="n">
-        <v>4</v>
-      </c>
-      <c r="H14" t="n">
-        <v>13</v>
-      </c>
-      <c r="I14" t="n">
-        <v>2</v>
-      </c>
-      <c r="J14" t="n">
-        <v>0.375</v>
-      </c>
-      <c r="K14" t="n">
-        <v>4</v>
-      </c>
-      <c r="L14" t="n">
-        <v>0.58064514</v>
-      </c>
-      <c r="M14" t="n">
-        <v>1</v>
       </c>
       <c r="N14" t="n">
         <v>6.230769</v>
@@ -3677,34 +3677,34 @@
         <v>8</v>
       </c>
       <c r="D15" t="n">
+        <v>38</v>
+      </c>
+      <c r="E15" t="n">
+        <v>5</v>
+      </c>
+      <c r="F15" t="n">
+        <v>14</v>
+      </c>
+      <c r="G15" t="n">
+        <v>1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0.3321033</v>
+      </c>
+      <c r="I15" t="n">
+        <v>10</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0.5222672</v>
+      </c>
+      <c r="K15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L15" t="n">
         <v>66</v>
       </c>
-      <c r="E15" t="n">
+      <c r="M15" t="n">
         <v>28</v>
-      </c>
-      <c r="F15" t="n">
-        <v>38</v>
-      </c>
-      <c r="G15" t="n">
-        <v>5</v>
-      </c>
-      <c r="H15" t="n">
-        <v>14</v>
-      </c>
-      <c r="I15" t="n">
-        <v>1</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0.3321033</v>
-      </c>
-      <c r="K15" t="n">
-        <v>10</v>
-      </c>
-      <c r="L15" t="n">
-        <v>0.5222672</v>
-      </c>
-      <c r="M15" t="n">
-        <v>3</v>
       </c>
       <c r="N15" t="n">
         <v>4.922652</v>
@@ -3744,34 +3744,34 @@
         <v>25</v>
       </c>
       <c r="D16" t="n">
-        <v>50</v>
+        <v>19</v>
       </c>
       <c r="E16" t="n">
-        <v>15</v>
+        <v>26</v>
       </c>
       <c r="F16" t="n">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="G16" t="n">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="H16" t="n">
-        <v>6</v>
+        <v>0.30232558</v>
       </c>
       <c r="I16" t="n">
         <v>21</v>
       </c>
       <c r="J16" t="n">
-        <v>0.30232558</v>
+        <v>0.35751295</v>
       </c>
       <c r="K16" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="L16" t="n">
-        <v>0.35751295</v>
+        <v>50</v>
       </c>
       <c r="M16" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="N16" t="n">
         <v>4.5</v>
@@ -3811,34 +3811,34 @@
         <v>19</v>
       </c>
       <c r="D17" t="n">
+        <v>26</v>
+      </c>
+      <c r="E17" t="n">
+        <v>14</v>
+      </c>
+      <c r="F17" t="n">
+        <v>9</v>
+      </c>
+      <c r="G17" t="n">
+        <v>9</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0.3196347</v>
+      </c>
+      <c r="I17" t="n">
+        <v>15</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0.43523315</v>
+      </c>
+      <c r="K17" t="n">
+        <v>11</v>
+      </c>
+      <c r="L17" t="n">
         <v>51</v>
       </c>
-      <c r="E17" t="n">
+      <c r="M17" t="n">
         <v>18</v>
-      </c>
-      <c r="F17" t="n">
-        <v>26</v>
-      </c>
-      <c r="G17" t="n">
-        <v>14</v>
-      </c>
-      <c r="H17" t="n">
-        <v>9</v>
-      </c>
-      <c r="I17" t="n">
-        <v>9</v>
-      </c>
-      <c r="J17" t="n">
-        <v>0.3196347</v>
-      </c>
-      <c r="K17" t="n">
-        <v>15</v>
-      </c>
-      <c r="L17" t="n">
-        <v>0.43523315</v>
-      </c>
-      <c r="M17" t="n">
-        <v>11</v>
       </c>
       <c r="N17" t="n">
         <v>4.1538463</v>
@@ -3878,34 +3878,34 @@
         <v>10</v>
       </c>
       <c r="D18" t="n">
+        <v>27</v>
+      </c>
+      <c r="E18" t="n">
+        <v>12</v>
+      </c>
+      <c r="F18" t="n">
+        <v>5</v>
+      </c>
+      <c r="G18" t="n">
+        <v>25</v>
+      </c>
+      <c r="H18" t="n">
+        <v>0.3318584</v>
+      </c>
+      <c r="I18" t="n">
+        <v>11</v>
+      </c>
+      <c r="J18" t="n">
+        <v>0.37810946</v>
+      </c>
+      <c r="K18" t="n">
+        <v>23</v>
+      </c>
+      <c r="L18" t="n">
         <v>53</v>
       </c>
-      <c r="E18" t="n">
+      <c r="M18" t="n">
         <v>20</v>
-      </c>
-      <c r="F18" t="n">
-        <v>27</v>
-      </c>
-      <c r="G18" t="n">
-        <v>12</v>
-      </c>
-      <c r="H18" t="n">
-        <v>5</v>
-      </c>
-      <c r="I18" t="n">
-        <v>25</v>
-      </c>
-      <c r="J18" t="n">
-        <v>0.3318584</v>
-      </c>
-      <c r="K18" t="n">
-        <v>11</v>
-      </c>
-      <c r="L18" t="n">
-        <v>0.37810946</v>
-      </c>
-      <c r="M18" t="n">
-        <v>23</v>
       </c>
       <c r="N18" t="n">
         <v>3.4394906</v>
@@ -3945,34 +3945,34 @@
         <v>1</v>
       </c>
       <c r="D19" t="n">
-        <v>39</v>
+        <v>50</v>
       </c>
       <c r="E19" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F19" t="n">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="H19" t="n">
-        <v>11</v>
+        <v>0.38339922</v>
       </c>
       <c r="I19" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J19" t="n">
-        <v>0.38339922</v>
+        <v>0.5414847</v>
       </c>
       <c r="K19" t="n">
         <v>2</v>
       </c>
       <c r="L19" t="n">
-        <v>0.5414847</v>
+        <v>39</v>
       </c>
       <c r="M19" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="N19" t="n">
         <v>3.9056604</v>
@@ -4012,34 +4012,34 @@
         <v>11</v>
       </c>
       <c r="D20" t="n">
+        <v>23</v>
+      </c>
+      <c r="E20" t="n">
+        <v>20</v>
+      </c>
+      <c r="F20" t="n">
+        <v>6</v>
+      </c>
+      <c r="G20" t="n">
+        <v>21</v>
+      </c>
+      <c r="H20" t="n">
+        <v>0.32765958</v>
+      </c>
+      <c r="I20" t="n">
+        <v>12</v>
+      </c>
+      <c r="J20" t="n">
+        <v>0.3809524</v>
+      </c>
+      <c r="K20" t="n">
+        <v>20</v>
+      </c>
+      <c r="L20" t="n">
         <v>57</v>
       </c>
-      <c r="E20" t="n">
+      <c r="M20" t="n">
         <v>21</v>
-      </c>
-      <c r="F20" t="n">
-        <v>23</v>
-      </c>
-      <c r="G20" t="n">
-        <v>20</v>
-      </c>
-      <c r="H20" t="n">
-        <v>6</v>
-      </c>
-      <c r="I20" t="n">
-        <v>21</v>
-      </c>
-      <c r="J20" t="n">
-        <v>0.32765958</v>
-      </c>
-      <c r="K20" t="n">
-        <v>12</v>
-      </c>
-      <c r="L20" t="n">
-        <v>0.3809524</v>
-      </c>
-      <c r="M20" t="n">
-        <v>20</v>
       </c>
       <c r="N20" t="n">
         <v>7.2</v>
@@ -4079,34 +4079,34 @@
         <v>7</v>
       </c>
       <c r="D21" t="n">
+        <v>31</v>
+      </c>
+      <c r="E21" t="n">
+        <v>9</v>
+      </c>
+      <c r="F21" t="n">
+        <v>12</v>
+      </c>
+      <c r="G21" t="n">
+        <v>4</v>
+      </c>
+      <c r="H21" t="n">
+        <v>0.35371178</v>
+      </c>
+      <c r="I21" t="n">
+        <v>5</v>
+      </c>
+      <c r="J21" t="n">
+        <v>0.502439</v>
+      </c>
+      <c r="K21" t="n">
+        <v>6</v>
+      </c>
+      <c r="L21" t="n">
         <v>50</v>
       </c>
-      <c r="E21" t="n">
+      <c r="M21" t="n">
         <v>15</v>
-      </c>
-      <c r="F21" t="n">
-        <v>31</v>
-      </c>
-      <c r="G21" t="n">
-        <v>9</v>
-      </c>
-      <c r="H21" t="n">
-        <v>12</v>
-      </c>
-      <c r="I21" t="n">
-        <v>4</v>
-      </c>
-      <c r="J21" t="n">
-        <v>0.35371178</v>
-      </c>
-      <c r="K21" t="n">
-        <v>5</v>
-      </c>
-      <c r="L21" t="n">
-        <v>0.502439</v>
-      </c>
-      <c r="M21" t="n">
-        <v>6</v>
       </c>
       <c r="N21" t="n">
         <v>3.6666667</v>
@@ -4146,34 +4146,34 @@
         <v>5</v>
       </c>
       <c r="D22" t="n">
+        <v>44</v>
+      </c>
+      <c r="E22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F22" t="n">
+        <v>11</v>
+      </c>
+      <c r="G22" t="n">
+        <v>5</v>
+      </c>
+      <c r="H22" t="n">
+        <v>0.34649122</v>
+      </c>
+      <c r="I22" t="n">
+        <v>6</v>
+      </c>
+      <c r="J22" t="n">
+        <v>0.5217391</v>
+      </c>
+      <c r="K22" t="n">
+        <v>5</v>
+      </c>
+      <c r="L22" t="n">
         <v>46</v>
       </c>
-      <c r="E22" t="n">
+      <c r="M22" t="n">
         <v>11</v>
-      </c>
-      <c r="F22" t="n">
-        <v>44</v>
-      </c>
-      <c r="G22" t="n">
-        <v>2</v>
-      </c>
-      <c r="H22" t="n">
-        <v>11</v>
-      </c>
-      <c r="I22" t="n">
-        <v>5</v>
-      </c>
-      <c r="J22" t="n">
-        <v>0.34649122</v>
-      </c>
-      <c r="K22" t="n">
-        <v>6</v>
-      </c>
-      <c r="L22" t="n">
-        <v>0.5217391</v>
-      </c>
-      <c r="M22" t="n">
-        <v>5</v>
       </c>
       <c r="N22" t="n">
         <v>3.5</v>
@@ -4213,34 +4213,34 @@
         <v>6</v>
       </c>
       <c r="D23" t="n">
-        <v>50</v>
+        <v>32</v>
       </c>
       <c r="E23" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F23" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="G23" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="H23" t="n">
-        <v>9</v>
+        <v>0.33474576</v>
       </c>
       <c r="I23" t="n">
         <v>9</v>
       </c>
       <c r="J23" t="n">
-        <v>0.33474576</v>
+        <v>0.48623854</v>
       </c>
       <c r="K23" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="L23" t="n">
-        <v>0.48623854</v>
+        <v>50</v>
       </c>
       <c r="M23" t="n">
-        <v>7</v>
+        <v>15</v>
       </c>
       <c r="N23" t="n">
         <v>4.0588236</v>
@@ -4280,34 +4280,34 @@
         <v>21</v>
       </c>
       <c r="D24" t="n">
+        <v>24</v>
+      </c>
+      <c r="E24" t="n">
+        <v>17</v>
+      </c>
+      <c r="F24" t="n">
+        <v>5</v>
+      </c>
+      <c r="G24" t="n">
+        <v>25</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.28636363</v>
+      </c>
+      <c r="I24" t="n">
+        <v>24</v>
+      </c>
+      <c r="J24" t="n">
+        <v>0.3546798</v>
+      </c>
+      <c r="K24" t="n">
+        <v>27</v>
+      </c>
+      <c r="L24" t="n">
         <v>57</v>
       </c>
-      <c r="E24" t="n">
+      <c r="M24" t="n">
         <v>21</v>
-      </c>
-      <c r="F24" t="n">
-        <v>24</v>
-      </c>
-      <c r="G24" t="n">
-        <v>17</v>
-      </c>
-      <c r="H24" t="n">
-        <v>5</v>
-      </c>
-      <c r="I24" t="n">
-        <v>25</v>
-      </c>
-      <c r="J24" t="n">
-        <v>0.28636363</v>
-      </c>
-      <c r="K24" t="n">
-        <v>24</v>
-      </c>
-      <c r="L24" t="n">
-        <v>0.3546798</v>
-      </c>
-      <c r="M24" t="n">
-        <v>27</v>
       </c>
       <c r="N24" t="n">
         <v>3.8823528</v>
@@ -4347,34 +4347,34 @@
         <v>14</v>
       </c>
       <c r="D25" t="n">
+        <v>21</v>
+      </c>
+      <c r="E25" t="n">
+        <v>23</v>
+      </c>
+      <c r="F25" t="n">
+        <v>8</v>
+      </c>
+      <c r="G25" t="n">
+        <v>12</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.31016043</v>
+      </c>
+      <c r="I25" t="n">
+        <v>19</v>
+      </c>
+      <c r="J25" t="n">
+        <v>0.45238096</v>
+      </c>
+      <c r="K25" t="n">
+        <v>9</v>
+      </c>
+      <c r="L25" t="n">
         <v>33</v>
       </c>
-      <c r="E25" t="n">
+      <c r="M25" t="n">
         <v>3</v>
-      </c>
-      <c r="F25" t="n">
-        <v>21</v>
-      </c>
-      <c r="G25" t="n">
-        <v>23</v>
-      </c>
-      <c r="H25" t="n">
-        <v>8</v>
-      </c>
-      <c r="I25" t="n">
-        <v>12</v>
-      </c>
-      <c r="J25" t="n">
-        <v>0.31016043</v>
-      </c>
-      <c r="K25" t="n">
-        <v>19</v>
-      </c>
-      <c r="L25" t="n">
-        <v>0.45238096</v>
-      </c>
-      <c r="M25" t="n">
-        <v>9</v>
       </c>
       <c r="N25" t="n">
         <v>3.642857</v>
@@ -4414,34 +4414,34 @@
         <v>30</v>
       </c>
       <c r="D26" t="n">
-        <v>48</v>
+        <v>15</v>
       </c>
       <c r="E26" t="n">
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="F26" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="G26" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H26" t="n">
-        <v>4</v>
+        <v>0.26020408</v>
       </c>
       <c r="I26" t="n">
         <v>28</v>
       </c>
       <c r="J26" t="n">
-        <v>0.26020408</v>
+        <v>0.24855492</v>
       </c>
       <c r="K26" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="L26" t="n">
-        <v>0.24855492</v>
+        <v>48</v>
       </c>
       <c r="M26" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="N26" t="n">
         <v>2.8333333</v>
@@ -4481,34 +4481,34 @@
         <v>4</v>
       </c>
       <c r="D27" t="n">
+        <v>30</v>
+      </c>
+      <c r="E27" t="n">
+        <v>11</v>
+      </c>
+      <c r="F27" t="n">
+        <v>4</v>
+      </c>
+      <c r="G27" t="n">
+        <v>28</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.37815127</v>
+      </c>
+      <c r="I27" t="n">
+        <v>3</v>
+      </c>
+      <c r="J27" t="n">
+        <v>0.42364532</v>
+      </c>
+      <c r="K27" t="n">
+        <v>14</v>
+      </c>
+      <c r="L27" t="n">
         <v>27</v>
       </c>
-      <c r="E27" t="n">
+      <c r="M27" t="n">
         <v>1</v>
-      </c>
-      <c r="F27" t="n">
-        <v>30</v>
-      </c>
-      <c r="G27" t="n">
-        <v>11</v>
-      </c>
-      <c r="H27" t="n">
-        <v>4</v>
-      </c>
-      <c r="I27" t="n">
-        <v>28</v>
-      </c>
-      <c r="J27" t="n">
-        <v>0.37815127</v>
-      </c>
-      <c r="K27" t="n">
-        <v>3</v>
-      </c>
-      <c r="L27" t="n">
-        <v>0.42364532</v>
-      </c>
-      <c r="M27" t="n">
-        <v>14</v>
       </c>
       <c r="N27" t="n">
         <v>6.0576925</v>
@@ -4548,34 +4548,34 @@
         <v>14</v>
       </c>
       <c r="D28" t="n">
+        <v>19</v>
+      </c>
+      <c r="E28" t="n">
+        <v>26</v>
+      </c>
+      <c r="F28" t="n">
+        <v>5</v>
+      </c>
+      <c r="G28" t="n">
+        <v>25</v>
+      </c>
+      <c r="H28" t="n">
+        <v>0.317757</v>
+      </c>
+      <c r="I28" t="n">
+        <v>16</v>
+      </c>
+      <c r="J28" t="n">
+        <v>0.36979166</v>
+      </c>
+      <c r="K28" t="n">
+        <v>25</v>
+      </c>
+      <c r="L28" t="n">
         <v>45</v>
       </c>
-      <c r="E28" t="n">
+      <c r="M28" t="n">
         <v>10</v>
-      </c>
-      <c r="F28" t="n">
-        <v>19</v>
-      </c>
-      <c r="G28" t="n">
-        <v>26</v>
-      </c>
-      <c r="H28" t="n">
-        <v>5</v>
-      </c>
-      <c r="I28" t="n">
-        <v>25</v>
-      </c>
-      <c r="J28" t="n">
-        <v>0.317757</v>
-      </c>
-      <c r="K28" t="n">
-        <v>16</v>
-      </c>
-      <c r="L28" t="n">
-        <v>0.36979166</v>
-      </c>
-      <c r="M28" t="n">
-        <v>25</v>
       </c>
       <c r="N28" t="n">
         <v>3.3529413</v>
@@ -4615,34 +4615,34 @@
         <v>9</v>
       </c>
       <c r="D29" t="n">
+        <v>24</v>
+      </c>
+      <c r="E29" t="n">
+        <v>17</v>
+      </c>
+      <c r="F29" t="n">
+        <v>7</v>
+      </c>
+      <c r="G29" t="n">
+        <v>16</v>
+      </c>
+      <c r="H29" t="n">
+        <v>0.32286996</v>
+      </c>
+      <c r="I29" t="n">
+        <v>14</v>
+      </c>
+      <c r="J29" t="n">
+        <v>0.41747573</v>
+      </c>
+      <c r="K29" t="n">
+        <v>15</v>
+      </c>
+      <c r="L29" t="n">
         <v>52</v>
       </c>
-      <c r="E29" t="n">
+      <c r="M29" t="n">
         <v>19</v>
-      </c>
-      <c r="F29" t="n">
-        <v>24</v>
-      </c>
-      <c r="G29" t="n">
-        <v>17</v>
-      </c>
-      <c r="H29" t="n">
-        <v>7</v>
-      </c>
-      <c r="I29" t="n">
-        <v>16</v>
-      </c>
-      <c r="J29" t="n">
-        <v>0.32286996</v>
-      </c>
-      <c r="K29" t="n">
-        <v>14</v>
-      </c>
-      <c r="L29" t="n">
-        <v>0.41747573</v>
-      </c>
-      <c r="M29" t="n">
-        <v>15</v>
       </c>
       <c r="N29" t="n">
         <v>5.890909</v>
@@ -4682,34 +4682,34 @@
         <v>22</v>
       </c>
       <c r="D30" t="n">
+        <v>23</v>
+      </c>
+      <c r="E30" t="n">
+        <v>20</v>
+      </c>
+      <c r="F30" t="n">
+        <v>8</v>
+      </c>
+      <c r="G30" t="n">
+        <v>12</v>
+      </c>
+      <c r="H30" t="n">
+        <v>0.26256984</v>
+      </c>
+      <c r="I30" t="n">
+        <v>27</v>
+      </c>
+      <c r="J30" t="n">
+        <v>0.43786982</v>
+      </c>
+      <c r="K30" t="n">
+        <v>10</v>
+      </c>
+      <c r="L30" t="n">
         <v>36</v>
       </c>
-      <c r="E30" t="n">
+      <c r="M30" t="n">
         <v>5</v>
-      </c>
-      <c r="F30" t="n">
-        <v>23</v>
-      </c>
-      <c r="G30" t="n">
-        <v>20</v>
-      </c>
-      <c r="H30" t="n">
-        <v>8</v>
-      </c>
-      <c r="I30" t="n">
-        <v>12</v>
-      </c>
-      <c r="J30" t="n">
-        <v>0.26256984</v>
-      </c>
-      <c r="K30" t="n">
-        <v>27</v>
-      </c>
-      <c r="L30" t="n">
-        <v>0.43786982</v>
-      </c>
-      <c r="M30" t="n">
-        <v>10</v>
       </c>
       <c r="N30" t="n">
         <v>4.2954545</v>
@@ -4749,34 +4749,34 @@
         <v>17</v>
       </c>
       <c r="D31" t="n">
+        <v>24</v>
+      </c>
+      <c r="E31" t="n">
+        <v>17</v>
+      </c>
+      <c r="F31" t="n">
+        <v>7</v>
+      </c>
+      <c r="G31" t="n">
+        <v>16</v>
+      </c>
+      <c r="H31" t="n">
+        <v>0.29186603</v>
+      </c>
+      <c r="I31" t="n">
+        <v>22</v>
+      </c>
+      <c r="J31" t="n">
+        <v>0.40625</v>
+      </c>
+      <c r="K31" t="n">
+        <v>18</v>
+      </c>
+      <c r="L31" t="n">
         <v>37</v>
       </c>
-      <c r="E31" t="n">
+      <c r="M31" t="n">
         <v>6</v>
-      </c>
-      <c r="F31" t="n">
-        <v>24</v>
-      </c>
-      <c r="G31" t="n">
-        <v>17</v>
-      </c>
-      <c r="H31" t="n">
-        <v>7</v>
-      </c>
-      <c r="I31" t="n">
-        <v>16</v>
-      </c>
-      <c r="J31" t="n">
-        <v>0.29186603</v>
-      </c>
-      <c r="K31" t="n">
-        <v>22</v>
-      </c>
-      <c r="L31" t="n">
-        <v>0.40625</v>
-      </c>
-      <c r="M31" t="n">
-        <v>18</v>
       </c>
       <c r="N31" t="n">
         <v>4.326923</v>

</xml_diff>